<commit_message>
PCA exploration for traits selection Updated scripts handling matrices
</commit_message>
<xml_diff>
--- a/results/LM CM x microclimatic gradients.xlsx
+++ b/results/LM CM x microclimatic gradients.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/Germination_drivers/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laptop\OneDrive - Universidad de Oviedo\IMIB\Softwares\GitHub\Germination_drivers\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{504918EE-862F-48CD-8BA5-2925155F0067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B66E660-1742-461A-9349-DB362CEF27A9}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B9778E14-6B2B-478F-9007-B73E2D75E56E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="transformed variables" sheetId="1" r:id="rId1"/>
+    <sheet name="transf variables_oct update" sheetId="1" r:id="rId1"/>
+    <sheet name="transformed variables_april" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="59">
   <si>
     <t>MEDITERRANEAN</t>
   </si>
@@ -783,13 +783,25 @@
       </rPr>
       <t>GDD                      + seed mass</t>
     </r>
+  </si>
+  <si>
+    <t>Leaf_area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no Log </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDMC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLA </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -834,7 +846,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -857,14 +869,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -873,9 +902,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,433 +1248,807 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECCEAD31-F739-4785-B83A-6721F2E617DB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" customWidth="1"/>
-    <col min="13" max="13" width="12.85546875" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.375" customWidth="1"/>
+    <col min="3" max="3" width="11.125" customWidth="1"/>
+    <col min="4" max="4" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.125" customWidth="1"/>
+    <col min="6" max="6" width="13.375" customWidth="1"/>
+    <col min="7" max="7" width="12.375" customWidth="1"/>
+    <col min="8" max="8" width="12.875" customWidth="1"/>
+    <col min="9" max="9" width="15.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="24" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="23.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="18">
       <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" ht="14.25" customHeight="1">
       <c r="A3" s="2"/>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="L3" s="9"/>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="J4" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="42.75">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2" t="s">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2" t="s">
+      <c r="H5" s="3"/>
+      <c r="I5" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+    </row>
+    <row r="6" spans="1:12" ht="43.5">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2" t="s">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-    </row>
-    <row r="7" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+    </row>
+    <row r="7" spans="1:12" ht="43.5">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2" t="s">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-    </row>
-    <row r="8" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+    </row>
+    <row r="8" spans="1:12" ht="43.5">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-    </row>
-    <row r="10" spans="1:14" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:12" ht="18">
       <c r="A10" s="2"/>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" ht="15" customHeight="1">
       <c r="A11" s="2"/>
-      <c r="B11" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4" t="s">
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="L11" s="9"/>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="G12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="H12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="I12" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="J12" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="44.25">
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2" t="s">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="H13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N13" s="2"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I13" s="3"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-    </row>
-    <row r="15" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+    </row>
+    <row r="15" spans="1:12" ht="43.5">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2" t="s">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2" t="s">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="G15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2" t="s">
+      <c r="H15" s="3"/>
+      <c r="I15" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+    </row>
+    <row r="16" spans="1:12" ht="44.25">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="I16" s="3"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="F3:J3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="F11:J11"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="85" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:Q16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.625" customWidth="1"/>
+    <col min="3" max="3" width="9.75" customWidth="1"/>
+    <col min="4" max="4" width="10.125" customWidth="1"/>
+    <col min="5" max="5" width="10.875" customWidth="1"/>
+    <col min="6" max="6" width="7.375" customWidth="1"/>
+    <col min="7" max="7" width="10.375" customWidth="1"/>
+    <col min="8" max="8" width="11.125" customWidth="1"/>
+    <col min="9" max="9" width="11.625" customWidth="1"/>
+    <col min="10" max="10" width="11.125" customWidth="1"/>
+    <col min="11" max="11" width="13.375" customWidth="1"/>
+    <col min="12" max="12" width="12.375" customWidth="1"/>
+    <col min="13" max="13" width="12.875" customWidth="1"/>
+    <col min="14" max="14" width="15.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="23.25">
+      <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="18">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="3"/>
+      <c r="B3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+    </row>
+    <row r="5" spans="1:17" ht="42.75">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="43.5">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+    </row>
+    <row r="7" spans="1:17" ht="43.5">
+      <c r="A7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+    </row>
+    <row r="8" spans="1:17" ht="43.5">
+      <c r="A8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" spans="1:17" ht="18">
+      <c r="A10" s="3"/>
+      <c r="B10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+    </row>
+    <row r="11" spans="1:17" ht="15" customHeight="1">
+      <c r="A11" s="3"/>
+      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+    </row>
+    <row r="12" spans="1:17">
+      <c r="A12" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="44.25">
+      <c r="A13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:17">
+      <c r="A14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:17" ht="43.5">
+      <c r="A15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="44.25">
+      <c r="A16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2" t="s">
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2" t="s">
+      <c r="L16" s="3"/>
+      <c r="M16" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="N16" s="2"/>
+      <c r="N16" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>